<commit_message>
Fix spreadsheets: show full YouTube URLs as visible clickable hyperlinks
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BPNpyGGfoMks39RbU3VXCG
</commit_message>
<xml_diff>
--- a/Comunicacao_Apresentacao_YouTube.xlsx
+++ b/Comunicacao_Apresentacao_YouTube.xlsx
@@ -58,7 +58,7 @@
     <font>
       <name val="Calibri"/>
       <color rgb="001155CC"/>
-      <sz val="9"/>
+      <sz val="8"/>
       <u val="single"/>
     </font>
     <font>
@@ -186,7 +186,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -204,7 +204,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -222,7 +222,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -240,7 +240,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -712,7 +712,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=NJlBdiTUL-8</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=MXKkXXYUxBc</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=aRIQgQxGpss</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=vgUUGM65xFs</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=gHXSwOTuseA</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=u1xRlsrfPyU</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=vfXQ18m_OsE</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=fPb1Ersu0pk</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=fntKY1Y0xGI</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=JkhA2cxeOaA</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=cTQHrNOlAUo</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=y8N8W0Q3RIk</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=2LABVbAgStA</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=WwaNX9HhJ_8</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=N05mgOlRfFg</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=tW3WDNjT6gk</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="C21" s="24" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=Z8wI6QvJEdk</t>
         </is>
       </c>
       <c r="D21" s="25" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=epKEXCHjp4M</t>
         </is>
       </c>
       <c r="D22" s="19" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="C23" s="24" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=JW8uwCbFCS0</t>
         </is>
       </c>
       <c r="D23" s="25" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>▶ Abrir Vídeo</t>
+          <t>https://www.youtube.com/watch?v=vhGsIAG1Boc</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">

</xml_diff>